<commit_message>
Update reports 2026-10-12 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-12.xlsx
+++ b/gex_pivot_levels_2026-10-12.xlsx
@@ -19,8 +19,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -573,12 +573,12 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>-$4.86M</t>
+          <t>-$4.17M</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+$11.52M</t>
+          <t>+$9.88M</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>-$9.43M</t>
+          <t>-$8.44M</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>+$15.48M</t>
+          <t>+$13.87M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -664,12 +664,12 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>+$5.61M</t>
+          <t>+$5.17M</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$63.19M</t>
+          <t>+$58.27M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -697,12 +697,12 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-$2.37M</t>
+          <t>-$2.22M</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>+$40.14M</t>
+          <t>+$37.55M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -730,12 +730,12 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>+$32.86M</t>
+          <t>+$31.32M</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>+$42.62M</t>
+          <t>+$40.63M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -796,12 +796,12 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>+$10.80M</t>
+          <t>+$11.00M</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>+$13.72M</t>
+          <t>+$13.96M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>+$36.64M</t>
+          <t>+$37.97M</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>+$41.83M</t>
+          <t>+$43.35M</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>+$27.84M</t>
+          <t>+$30.16M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$42.03M</t>
+          <t>+$45.54M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -891,12 +891,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>+$12.57M</t>
+          <t>+$14.37M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$13.10M</t>
+          <t>+$14.97M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2612,7 +2612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2696,24 +2696,24 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>4190.47</v>
+        <v>4188.05</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>88.5</v>
+        <v>381</v>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>+$8.27M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>-$1.83M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$8.38M</t>
+          <t>+$3.25M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -2723,30 +2723,30 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>4221.02</v>
+        <v>4190.47</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>384</v>
+        <v>88.5</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>+$3.27M</t>
+          <t>+$8.27M</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>+$3.36M</t>
+          <t>+$8.38M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -2762,10 +2762,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4243.01</v>
+        <v>4221.02</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
@@ -2774,45 +2774,41 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>+$335.93K</t>
+          <t>+$1.50M</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>+$577.67K</t>
+          <t>+$4.44M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>4254</v>
+        <v>4261.49</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>387</v>
+        <v>90</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>+$5.98M</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>-$253.77K</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$6.40M</t>
+          <t>+$15.69M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -2822,30 +2818,30 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>4261.49</v>
+        <v>4264.99</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>90</v>
+        <v>388</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>-$253.77K</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>+$6.25M</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>+$15.69M</t>
+          <t>+$6.36M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -2855,16 +2851,16 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>4275.99</v>
+        <v>4297.97</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -2873,45 +2869,41 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>+$334.20K</t>
+          <t>+$1.73M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$529.07K</t>
+          <t>+$1.73M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>4297.97</v>
+        <v>4332.52</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>391</v>
+        <v>91.5</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>+$1.51M</t>
+          <t>+$7.69M</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>+$1.51M</t>
+          <t>+$7.90M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -2926,110 +2918,106 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>4332.52</v>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>91.5</v>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="A10" s="2" t="n">
+        <v>4356.19</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>+$7.69M</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>+$7.90M</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>-$1.66M</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>+$4.59M</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>4403.54</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>+$2.53M</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>+$3.38M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>4356.19</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>92</v>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>4450.89</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>-$1.66M</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>+$4.59M</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>4403.54</v>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>93</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>+$2.53M</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>+$3.38M</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>+$796.63K</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>+$1.49M</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>4450.89</v>
+        <v>4498.24</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -3038,12 +3026,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>+$796.63K</t>
+          <t>+$475.12K</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$1.49M</t>
+          <t>+$5.06M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -3055,10 +3043,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>4498.24</v>
+        <v>4734.99</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
@@ -3067,12 +3055,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>+$475.12K</t>
+          <t>+$1.40M</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>+$5.06M</t>
+          <t>+$1.48M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -3082,37 +3070,8 @@
       </c>
       <c r="G14" s="3" t="inlineStr"/>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>4734.99</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>+$1.40M</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>+$1.48M</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G15"/>
+  <autoFilter ref="A1:G14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3124,7 +3083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3236,12 +3195,12 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>+$5.61M</t>
+          <t>+$5.17M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>+$63.19M</t>
+          <t>+$58.27M</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -3262,24 +3221,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>7859.21</v>
+        <v>7923.46</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>776</v>
+        <v>7850</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>+$10.47M</t>
+          <t>+$30.16M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>+$43.04M</t>
+          <t>+$45.54M</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3296,10 +3255,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>7893.46</v>
+        <v>7913.46</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>7820</v>
+        <v>7840</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
@@ -3308,12 +3267,12 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>+$32.86M</t>
+          <t>+$37.97M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>+$42.62M</t>
+          <t>+$43.35M</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -3334,24 +3293,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>7923.46</v>
+        <v>7859.21</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>7850</v>
+        <v>776</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>+$27.84M</t>
+          <t>+$10.47M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$42.03M</t>
+          <t>+$43.04M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3368,10 +3327,10 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7913.46</v>
+        <v>7893.46</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>7840</v>
+        <v>7820</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -3380,12 +3339,12 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>+$36.64M</t>
+          <t>+$31.32M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>+$41.83M</t>
+          <t>+$40.63M</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -3418,12 +3377,12 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>-$2.37M</t>
+          <t>-$2.22M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>+$40.14M</t>
+          <t>+$37.55M</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -3696,42 +3655,38 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
-        <v>7853.46</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>7780</v>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="B16" s="2" t="n">
+        <v>7948.46</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>7875</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>-$9.43M</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>+$15.48M</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>+$14.37M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>+$14.97M</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -3790,12 +3745,12 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>+$10.80M</t>
+          <t>+$11.00M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>+$13.72M</t>
+          <t>+$13.96M</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -3810,38 +3765,42 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
-        <v>7799.02</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>770</v>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>-$7.83M</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>+$13.46M</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
+      <c r="B19" s="5" t="n">
+        <v>7853.46</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>7780</v>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>-$8.44M</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>+$13.87M</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -3850,24 +3809,24 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7948.46</v>
+        <v>7799.02</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>7875</v>
+        <v>770</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>+$12.57M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>-$7.83M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+$13.10M</t>
+          <t>+$13.46M</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -3918,28 +3877,28 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>7823.46</v>
+        <v>2796.68</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>7750</v>
+        <v>278</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>-$4.86M</t>
+          <t>-$1.08M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>+$11.52M</t>
+          <t>+$10.68M</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -3950,38 +3909,42 @@
       <c r="H22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
-        <v>2796.68</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>278</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="B23" s="5" t="n">
+        <v>2846.98</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>283</v>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>-$1.08M</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>+$10.68M</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>+$8.62M</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>+$10.55M</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -3990,24 +3953,24 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>2846.98</v>
+        <v>2766.5</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>+$8.62M</t>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>-$6.61M</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>+$10.55M</t>
+          <t>+$10.32M</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -4017,73 +3980,69 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>2766.5</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>275</v>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>-$6.61M</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>+$10.32M</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>30937.39</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>744</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>-$8.23M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>+$10.11M</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>30937.39</v>
+        <v>7823.46</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>744</v>
+        <v>7750</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>-$8.23M</t>
+          <t>-$4.17M</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>+$10.11M</t>
+          <t>+$9.88M</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -4176,10 +4135,10 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>4254</v>
+        <v>4264.99</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -4188,12 +4147,12 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>+$5.98M</t>
+          <t>+$6.25M</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>+$6.40M</t>
+          <t>+$6.36M</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -4390,42 +4349,38 @@
       <c r="H34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B35" s="5" t="n">
-        <v>4403.54</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>93</v>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>+$2.53M</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>+$3.38M</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="B35" s="2" t="n">
+        <v>4221.02</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>384</v>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>+$1.50M</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>+$4.44M</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -4434,24 +4389,24 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>4221.02</v>
+        <v>4403.54</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>384</v>
+        <v>93</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>+$3.27M</t>
+          <t>+$2.53M</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>+$3.36M</t>
+          <t>+$3.38M</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -4472,24 +4427,24 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>4297.97</v>
+        <v>4188.05</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>391</v>
+        <v>381</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>+$1.51M</t>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>-$1.83M</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>+$1.51M</t>
+          <t>+$3.25M</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
@@ -4499,7 +4454,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4510,24 +4465,24 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>4450.89</v>
+        <v>4297.97</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>94</v>
+        <v>391</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>+$796.63K</t>
+          <t>+$1.73M</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>+$1.49M</t>
+          <t>+$1.73M</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -4544,10 +4499,10 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>4734.99</v>
+        <v>4450.89</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
@@ -4556,12 +4511,12 @@
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>+$1.40M</t>
+          <t>+$796.63K</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>+$1.48M</t>
+          <t>+$1.49M</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -4574,74 +4529,70 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>4734.99</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>+$1.40M</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>+$1.48M</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B41" s="2" t="n">
         <v>30731.85</v>
       </c>
-      <c r="C40" s="2" t="n">
+      <c r="C41" s="2" t="n">
         <v>739</v>
       </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>-$667.98K</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>+$1.19M</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>91.43000000000001</v>
-      </c>
-      <c r="C41" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
-          <t>+$476.07K</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>+$1.05M</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4654,24 +4605,24 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>82.28</v>
+        <v>91.43000000000001</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>-$980.97K</t>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>+$476.07K</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>+$999.64K</t>
+          <t>+$1.05M</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -4681,83 +4632,83 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>82.28</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>135</v>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>-$980.97K</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>+$999.64K</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B43" s="5" t="n">
+      <c r="B44" s="5" t="n">
         <v>31353.1</v>
       </c>
-      <c r="C43" s="5" t="n">
+      <c r="C44" s="5" t="n">
         <v>31000</v>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E44" s="9" t="inlineStr">
         <is>
           <t>+$143.61K</t>
         </is>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>+$579.06K</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n">
-        <v>4243.01</v>
-      </c>
-      <c r="C44" s="2" t="n">
-        <v>386</v>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>+$335.93K</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>+$577.67K</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4876,40 +4827,40 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>4275.99</v>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>389</v>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>+$334.20K</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>+$529.07K</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>88.38</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>+$32.81K</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>+$495.65K</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4920,24 +4871,24 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>88.38</v>
+        <v>85.33</v>
       </c>
       <c r="C49" s="5" t="n">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
-        <is>
-          <t>+$32.81K</t>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>-$369.05K</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>+$495.65K</t>
+          <t>+$430.63K</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
@@ -4947,81 +4898,81 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="n">
-        <v>85.33</v>
-      </c>
-      <c r="C50" s="5" t="n">
-        <v>140</v>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>-$369.05K</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>+$430.63K</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>31213.1</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>30860</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>-$108.71K</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>+$316.24K</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>31153.1</v>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>30800</v>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>-$134.34K</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>+$310.38K</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n">
-        <v>31213.1</v>
-      </c>
-      <c r="C51" s="2" t="n">
-        <v>30860</v>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>-$108.71K</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>+$316.24K</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -5030,10 +4981,10 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>31153.1</v>
+        <v>31053.1</v>
       </c>
       <c r="C52" s="5" t="n">
-        <v>30800</v>
+        <v>30700</v>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
@@ -5042,12 +4993,12 @@
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>-$134.34K</t>
+          <t>-$103.77K</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>+$310.38K</t>
+          <t>+$214.95K</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -5062,152 +5013,152 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n">
-        <v>31053.1</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>30700</v>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="B53" s="2" t="n">
+        <v>31223.1</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>30870</v>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>-$103.77K</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>+$214.95K</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>-$108.71K</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>+$207.53K</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B54" s="2" t="n">
-        <v>31223.1</v>
-      </c>
-      <c r="C54" s="2" t="n">
-        <v>30870</v>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="B54" s="5" t="n">
+        <v>31103.1</v>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>30750</v>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>-$108.71K</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>+$207.53K</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>-$121.06K</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>+$190.24K</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>97.52</v>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>+$170.99K</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>+$180.71K</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B55" s="5" t="n">
-        <v>31103.1</v>
-      </c>
-      <c r="C55" s="5" t="n">
-        <v>30750</v>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
+      <c r="B56" s="5" t="n">
+        <v>31183.1</v>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>30830</v>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr">
-        <is>
-          <t>-$121.06K</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>+$190.24K</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H55" s="6" t="inlineStr">
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>-$138.36K</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>+$168.00K</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="n">
-        <v>97.52</v>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>160</v>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>+$170.99K</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>+$180.71K</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -5216,24 +5167,24 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>31183.1</v>
+        <v>31083.1</v>
       </c>
       <c r="C57" s="5" t="n">
-        <v>30830</v>
+        <v>30730</v>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
-        <is>
-          <t>-$138.36K</t>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>+$132.49K</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>+$168.00K</t>
+          <t>+$164.61K</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
@@ -5243,7 +5194,7 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5254,10 +5205,10 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>31083.1</v>
+        <v>31283.1</v>
       </c>
       <c r="C58" s="5" t="n">
-        <v>30730</v>
+        <v>30930</v>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
@@ -5266,12 +5217,12 @@
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>+$132.49K</t>
+          <t>+$98.83K</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>+$164.61K</t>
+          <t>+$158.12K</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -5286,40 +5237,40 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B59" s="5" t="n">
-        <v>31283.1</v>
-      </c>
-      <c r="C59" s="5" t="n">
-        <v>30930</v>
-      </c>
-      <c r="D59" s="6" t="inlineStr">
+      <c r="B59" s="2" t="n">
+        <v>31078.1</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>30725</v>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E59" s="9" t="inlineStr">
-        <is>
-          <t>+$98.83K</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="inlineStr">
-        <is>
-          <t>+$158.12K</t>
-        </is>
-      </c>
-      <c r="G59" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H59" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>-$104.39K</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>+$136.50K</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5330,10 +5281,10 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>31078.1</v>
+        <v>31323.1</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>30725</v>
+        <v>30970</v>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
@@ -5342,24 +5293,20 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>-$104.39K</t>
+          <t>-$4.94K</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>+$136.50K</t>
+          <t>+$123.53K</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -5368,32 +5315,36 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>31323.1</v>
+        <v>31193.1</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>30970</v>
+        <v>30840</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>-$4.94K</t>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>+$69.18K</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>+$123.53K</t>
+          <t>+$118.59K</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -5402,10 +5353,10 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>31193.1</v>
+        <v>31303.1</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>30840</v>
+        <v>30950</v>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
@@ -5414,7 +5365,7 @@
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>+$69.18K</t>
+          <t>+$9.88K</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -5424,86 +5375,82 @@
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H62" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B63" s="2" t="n">
-        <v>31303.1</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>30950</v>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="B63" s="5" t="n">
+        <v>31128.1</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>30775</v>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>+$9.88K</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>+$118.59K</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr">
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>-$99.44K</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>+$116.74K</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>98.73999999999999</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>162</v>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>+$105.28K</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>+$109.18K</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H63" s="3" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="n">
-        <v>31128.1</v>
-      </c>
-      <c r="C64" s="5" t="n">
-        <v>30775</v>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>-$99.44K</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>+$116.74K</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -5512,10 +5459,10 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>98.73999999999999</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
@@ -5524,46 +5471,50 @@
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>+$105.28K</t>
+          <t>+$9.41K</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>+$109.18K</t>
+          <t>+$95.80K</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H65" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>92.65000000000001</v>
+        <v>31333.1</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>152</v>
+        <v>30980</v>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>+$9.41K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>-$29.65K</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>+$95.80K</t>
+          <t>+$88.94K</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -5584,36 +5535,32 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>31333.1</v>
+        <v>31403.1</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>30980</v>
+        <v>31050</v>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>-$29.65K</t>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>+$44.16K</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>+$88.94K</t>
+          <t>+$84.31K</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -5622,10 +5569,10 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>31403.1</v>
+        <v>31123.1</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>31050</v>
+        <v>30770</v>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
@@ -5634,46 +5581,50 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>+$44.16K</t>
+          <t>+$21.62K</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>+$84.31K</t>
+          <t>+$64.85K</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H68" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>31123.1</v>
+        <v>82.89</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>30770</v>
+        <v>136</v>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>+$21.62K</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>-$44.38K</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>+$64.85K</t>
+          <t>+$50.58K</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -5690,28 +5641,28 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>82.89</v>
+        <v>31173.1</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>136</v>
+        <v>30820</v>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>-$44.38K</t>
+          <t>-$9.88K</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>+$50.58K</t>
+          <t>+$49.41K</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -5732,24 +5683,24 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>31173.1</v>
+        <v>31278.1</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>30820</v>
+        <v>30925</v>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>-$9.88K</t>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>+$5.25K</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>+$49.41K</t>
+          <t>+$47.25K</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -5759,7 +5710,7 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5770,24 +5721,24 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>31278.1</v>
+        <v>31133.1</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>30925</v>
+        <v>30780</v>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E72" s="8" t="inlineStr">
-        <is>
-          <t>+$5.25K</t>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>-$32.43K</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>+$47.25K</t>
+          <t>+$41.69K</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -5797,7 +5748,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5808,10 +5759,10 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>31133.1</v>
+        <v>31063.1</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>30780</v>
+        <v>30710</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
@@ -5820,12 +5771,12 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>-$32.43K</t>
+          <t>-$11.12K</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>+$41.69K</t>
+          <t>+$11.12K</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -5839,46 +5790,8 @@
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="n">
-        <v>31063.1</v>
-      </c>
-      <c r="C74" s="2" t="n">
-        <v>30710</v>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>-$11.12K</t>
-        </is>
-      </c>
-      <c r="F74" s="3" t="inlineStr">
-        <is>
-          <t>+$11.12K</t>
-        </is>
-      </c>
-      <c r="G74" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H74" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H74"/>
+  <autoFilter ref="A1:H73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>